<commit_message>
Add DeploymentUI and QuestBoardUI scripts for unit deployment and quest selection
- Implemented DeploymentUI.client.lua to manage unit deployment phase, including tile highlights, enemy tokens, and player unit roster.
- Created QuestBoardUI.client.lua to display quest options and handle quest selection from the server.
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Game_Rules.xlsx
+++ b/docs/CTRBLXAI_Game_Rules.xlsx
@@ -38,6 +38,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 Persistent HP MP" sheetId="29" state="visible" r:id="rId29"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 Item Affix Names" sheetId="30" state="visible" r:id="rId30"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 Unit Progression" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22 Economy Framework" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23 Materials System" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01 Project Identity'!$A$1:$D$79</definedName>
@@ -56,7 +58,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,8 +81,18 @@
     <font>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002F5496"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +117,12 @@
         <bgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+        <bgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -124,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -136,6 +154,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -503,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D105"/>
+  <dimension ref="A1:D108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2640,6 +2667,40 @@
       <c r="C105" t="inlineStr">
         <is>
           <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>RNG scope</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>No hit/miss, dodge, or debuff infliction RNG. Combat resolution is deterministic. RNG is used for procedural generation: maps, item bonuses, loot drops, enemy spawns, recruit pools, terrain placement.</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Equipment Downgrade</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Downgrading equipment is FREE. No compensation. Purpose: reduce item level for lower-level unit equip. Upgrading costs gold/materials (blacksmith design pending).</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
         </is>
       </c>
     </row>
@@ -42061,7 +42122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42074,7 +42135,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kill-based XP + procedural objectives. Linear ramp: XP to level = 500 + (Level × 20). L99 cap at launch. Evolutions post-launch.</t>
+          <t>Kill-based XP + procedural objectives. Linear ramp: XP to level = 500 + (Level × 20). Defeat/victory reward rules. Dispatch. Bench rate 65%.</t>
         </is>
       </c>
     </row>
@@ -42553,12 +42614,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>50% of battle XP. Prevents permanent roster gaps.</t>
+          <t>65% of battle XP. Prevents permanent roster gaps. Benched units stay viable without mandatory rotation.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Locked</t>
+          <t>Locked — updated from 50% based on simulation v2</t>
         </is>
       </c>
     </row>
@@ -43103,12 +43164,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Dispatched units earn flat XP based on dispatch difficulty × duration. Unit unavailable for N battles.</t>
+          <t>Dispatched units earn flat XP based on dispatch difficulty × duration. Unit unavailable for N battles. Dispatch appears as a quest on the quest board but does NOT initiate a battle. Player selects units and sends them; they return after the specified duration with rewards.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Locked direction</t>
+          <t>Locked direction — dispatch is quest board activity, not battle</t>
         </is>
       </c>
     </row>
@@ -43172,7 +43233,6 @@
           <t>Slice 6 owns XP system implementation. Base formula can work without Slice 5. Procedural objectives need Slice 5 map spawns.</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -43190,7 +43250,6 @@
           <t>Slice 5: procedural maps for objectives. Slice 8: quest board, dispatch, exploration. Daily/seasonal events: separate reward systems, may grant XP as part of reward.</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -43365,6 +43424,2136 @@
       <c r="D62" t="inlineStr">
         <is>
           <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Defeat Rewards</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Enemy kill XP</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>XP from enemies defeated during battle is retained even on wipeout. Per-kill XP accumulates during battle and is awarded regardless of outcome.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Defeat Rewards</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Enemy loot drops</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Defeated enemies can trigger loot drops during battle. On wipeout: all loot drops are LOST. Only victory commits loot to inventory.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Defeat Rewards</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Gold on wipeout</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>On wipeout: player keeps 50% of gold earned from enemy kills during the battle. Other 50% is lost.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Defeat Rewards</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Quest rewards on defeat</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Quest rewards CANNOT be obtained on defeat. Quest progress is NOT advanced. The quest remains incomplete.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Defeat Rewards</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Guild XP penalty</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Wipeout or escape penalizes Guild XP. Exact penalty formula pending design. Direction: reduced or zero Guild XP from failed battles, possible negative Guild XP modifier for consecutive failures.</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Locked direction — exact formula pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Defeat Rewards</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Escape</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Escaping a battle follows the same reward rules as wipeout: keep kill XP, keep 50% gold, lose all loot, no quest progress, Guild XP penalty.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Defeat Rewards</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Persistent HP/MP on defeat</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Persistent HP/MP loss still applies on defeat. Units end battle at their current HP/MP. KO'd units follow KO recovery rules. No post-battle 35% recovery on defeat.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Victory Rewards</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Victory: 100% kill XP + 100% gold + all loot committed + quest progress + quest rewards + full Guild XP + post-battle 35% recovery.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Gold Sources</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Design Principle</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Basics always affordable. Everything at once is impossible. Free player covers necessities (~69% of income) with surplus for partial luxury progression.</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Gold Sources</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gold Formula</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gold = Base Gold × (1 + Enemy Level / 100). Scales at half the rate of XP (Level/100 vs Level/50) — intentional scarcity.</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Gold Sources</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gold — Grunt</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Base Gold = 8</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Gold Sources</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gold — Veteran</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Base Gold = 14</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Gold Sources</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gold — Elite</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Base Gold = 25</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Gold Sources</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gold — Boss</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Base Gold = 50</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Gold Sources</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gold — Overleveled Penalty</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Same bands as XP: gap ≤5 ×1.0, 6-10 ×0.75, 11-15 ×0.50, 16-20 ×0.25, 21+ ×0.10. Underleveled content gives NO bonus gold (prevents gold farming in hard content).</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Gold Sources</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Battle Completion Gold</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Base × (1 + Map Level / 50). Normal = 30, Elite = 50, Boss = 100, Survive/Protect = 40, Exploration = 25.</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Gold Sources</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Quest Reward Gold</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Base × (1 + Recommended Level / 40). Shown upfront before acceptance. Normal = 50, Elite = 80, Boss = 150, Exploration = 120, Dispatch = 40.</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Gold Sources</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Fortune Gold Multiplier</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>1 + 0.50 × Normalized Expedition Fortune. Max theoretical ×1.50. Applies to expedition-generated gold only.</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Locked — see loot_progression table</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Item Value</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Base Value by Slot</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>1H = 100, 2H = 150, Off-Hand = 60, Body = 80, Head = 60, Gloves = 50, Feet = 50, Accessory = 70.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Item Value</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Rarity Multiplier</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Broken = 0.1, Common = 1.0, Uncommon = 1.5, Rare = 2.5, Epic = 4.0, Legendary = 7.0, Mythic = 12.0, Transcendent = 20.0, Unique = 15.0.</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Item Value</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Level Multiplier</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>1 + (Item Level - 1) × 0.02. L1 = ×1.00, L50 = ×1.98, L99 = ×2.96.</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Item Value</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Sell Value Formula</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>floor(Base Value × Rarity Mult × Level Mult × 0.25). Supplementary income source (~6% of total income).</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Shop</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Shop Price Formula</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>round(Base Value × Rarity Mult × Level Mult × 4.0). Shop Markup = ×4.0.</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Shop</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Buy/Sell Ratio</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>16:1. Shop markup ×4.0 / Sell rate ×0.25. No profitable buy-sell loops.</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Shop</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Purchasing Power Stability</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>A level-appropriate Common weapon costs 2.5-2.7 battles at ANY level. Stable purchasing power across the full game.</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Locked — verified by simulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Shop</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Shop Stock</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Shops sell Common and Uncommon items up to current Map Level. Rare+ items are NOT available in shops — loot or blacksmith only. Merchant stock rotation rules pending.</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Locked direction — rotation details pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Blacksmith</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade Gold Cost Formula</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>floor(Base Value × Rarity Mult × 0.30 × (1 + Target Level / 25)). Per level. Plus materials (separate design).</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Locked — materials system pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Blacksmith</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Upgrade Cost Feel</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Rare weapon +30 levels ≈ 4 battles. Legendary weapon +25 levels ≈ 12 battles. Primary gold sink (~43% of lifetime income).</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Locked — verified by simulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Blacksmith</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Downgrade</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Free. No gold, materials, or compensation. Reduces item level so lower-level units can equip it.</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Fee Formula</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>200 + (Unit Level × 15) + Quality Premium. Standard = +0, Quality = +300, Elite = +800.</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Fee Feel</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>L1 Standard = 215g (1.3 battles). L50 Standard = 950g (3.1 battles). L50 Elite = 1750g (5.8 battles). Small portion of total spend (~2%).</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Locked — verified by simulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Inventory Maintenance</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Threshold</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>50 items. Items beyond threshold incur per-visit maintenance cost.</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Locked — tunable during testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Inventory Maintenance</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Cost Formula</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>min(Excess Items × 5, 200) gold per base visit. Excess = max(0, Item Count - 50).</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Locked — cap and per-item rate tunable</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Dispatch</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>50 gold per dispatch mission. Base 3 concurrent slots.</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Consumables</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Pricing Direction</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Individual consumable prices pending. Average ~50g per consumable. ~6% of lifetime income.</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Locked direction — individual prices pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Guild Facilities</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Long-term gold sink. Luxury progression (~44% of lifetime income). Cannot fully complete L1→L99 on free income alone — creates endgame engagement.</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Locked direction — individual facility costs pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Guild Facilities</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Estimated Curve</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>500 + (Guild Level × 200) per facility level. L1→L25 total ≈ 77,500g. Exact per-facility costs pending.</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Placeholder — pending Slice 8 design</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Robux Convenience</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Design Principle</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Convenience boosts only. No exclusive power. A boosted player with the same gear at the same level has zero combat advantage over a free player.</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Robux Convenience</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Gold Boost</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>+25% battle gold. Time-limited (24h / 7d / 30d). Moves lifetime expense ratio from 113% to 90% — makes guild facilities reachable without trivializing choices.</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>Robux Convenience</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>XP Boost</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>+25% battle XP. Time-limited (24h / 7d / 30d).</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Robux Convenience</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Inventory Expansion</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>+25 item threshold per purchase. Permanent. Reduces maintenance costs.</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>Robux Convenience</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Dispatch Slot</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>+1 concurrent dispatch slot (base 3, max 6). Permanent.</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>Robux Convenience</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Cosmetics</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Unit skins, HQ decoration, portraits, name changes. Permanent. No gameplay impact.</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>Robux Convenience</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Robux CANNOT Buy</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>Equipment, stats, levels, skill/augment/doctrine cards, materials, gold directly, exclusive content, rarity upgrades, recruitment shortcuts, combat advantage of any kind.</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>Robux Convenience</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Robux Price Points</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Pending Roblox marketplace research.</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>Economy Phases</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>L1-20 (Early)</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Gold flows freely. Buy basic gear, recruit early. Blacksmith affordable. Feels generous — hooks the player.</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Locked — verified by simulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>Economy Phases</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>L20-50 (Mid)</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Meaningful choices emerge. Upgrade or buy? Which unit? Guild facilities start competing for gold.</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Locked — verified by simulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>Economy Phases</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>L50-80 (Late)</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Tight. Legendary upgrades expensive. Must loot-hunt for Rare/Epic drops to reduce shop dependence.</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>Locked — verified by simulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>Economy Phases</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>L80-99 (Endgame)</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Scarcity. Guild facilities vs final gear upgrades. Gold Boost feels genuinely helpful, not mandatory.</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>Locked — verified by simulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>Simulation Benchmarks</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>Lifetime Income (L1→L99, ~547 battles)</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Battle gold ~165,000g + sell income ~10,800g = ~175,800g total.</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>Simulation Benchmarks</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Necessities Cost</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>~121,000g (69% of income). Recruitment + shop + blacksmith + consumables + ongoing.</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>Simulation Benchmarks</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Luxuries Cost</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>~78,000g (44% of income). Guild facilities. Cannot complete everything — intentional.</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>Simulation Benchmarks</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Free Player</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Covers all basics. Guild facilities up to ~L18 before deficit.</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>Simulation Benchmarks</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>Boosted Player (+25%)</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Covers basics + guild to ~L22. Expense ratio 90%.</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Material Tiers</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Design Principle</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>5 generic tiers, one material type per tier. No element-specific or slot-specific materials. The tier alone gates difficulty. Prevents frustrating RNG ('I need Fire Shards but only get Ice Shards').</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Material Tiers</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>T1 — Rough Fragment</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Gray. Drops from L1-25 content. Common drops, early chests.</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Material Tiers</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>T2 — Refined Shard</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Green. Drops from L20-50 content. Mid-game drops, quests.</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Material Tiers</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>T3 — Polished Core</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Blue. Drops from L40-70 content. Elite encounters, late-mid drops.</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Material Tiers</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>T4 — Pristine Crystal</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Purple. Drops from L60-90 content. Boss encounters, endgame drops.</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Material Tiers</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>T5 — Ethereal Essence</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Gold. Drops from L80-99 content. Daily events (only reliable source), rare L80+ boss drops, L90+ elite encounters.</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Drop Sources</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Normal Enemy Kill</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>20% chance per kill. 1 material. Tier based on enemy level range. Primary source (~1.6 per battle from 8 enemies).</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Drop Sources</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Elite Encounter</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>75% chance (1 guaranteed if rewarded). 2-3 materials. Tier = enemy level range.</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Drop Sources</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Boss Encounter</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>100% guaranteed. 3-5 materials. Tier = boss level range.</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Drop Sources</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Treasure Chest</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>100% on Interact. 1-2 materials + other loot.</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Locked — already in objects_encounters</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Drop Sources</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Quest Reward</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Shown upfront before acceptance. Varies by quest type and recommended level.</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Drop Sources</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Dispatch Reward</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Shown upfront. 1-3 materials, lower tier than current content.</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Drop Sources</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Daily Event</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>100% event reward. T5 Ethereal Essence exclusively. Only reliable T5 source.</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Drop Sources</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Destroyed Objects</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>30% chance with Salvager's Cap passive. 1 material.</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Locked — already in nonweapon_equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Drop Sources</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Average Per Battle</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>~2.6 materials per battle total (kills 1.6 + quest 0.5 + chest 0.3 + elite/boss 0.2).</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Locked — verified by simulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Drop Tier Rules</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Tier Assignment</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Material tier dropped matches content level range: L1-20 → T1, L21-40 → T2, L41-60 → T3, L61-80 → T4, L81-99 → T5.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Drop Tier Rules</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Overlap Handling</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Overlapping level ranges (e.g. L20 content) weighted toward lower tier.</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Drop Tier Rules</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>T5 Restriction</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>T5 Ethereal Essence ONLY from: daily events, L80+ boss encounters, and L90+ elite encounters. No other source.</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Drop Tier Rules</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Fortune Exclusion</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Fortune does NOT affect material drop rate, quantity, or tier. Materials are deterministic progression, not luck-gated.</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Locked — per loot_progression rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Blacksmith Recipes</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade Recipe</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Each upgrade level requires Gold (from economy_framework) + Materials. Material tier = based on target item level. Material quantity = based on item rarity.</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Blacksmith Recipes</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Tier by Target Level</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Target L1-20: T1. Target L21-40: T2. Target L41-60: T3. Target L61-80: T4. Target L81-99: T5.</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Blacksmith Recipes</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Quantity by Rarity</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Common = 1/level, Uncommon = 1/level, Rare = 2/level, Epic = 3/level, Legendary = 4/level, Mythic = 5/level, Transcendent = 6/level.</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Blacksmith Recipes</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Example — Rare 1H L50→L55</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Gold: 1,170g + Materials: 10× T3 Polished Core (5 levels × 2/level).</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Blacksmith Recipes</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Example — Legendary 1H L65→L90</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Gold: ~16,500g + Materials: 60× T4 Pristine Crystal (15 levels × 4/level for L66-80) + 40× T5 Ethereal Essence (10 levels × 4/level for L81-90).</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Material Conversion</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Conversion Formula</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>3× lower tier → 1× next tier. One-way, lossy. Available at Blacksmith facility.</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Material Conversion</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Prevents hoarding of low-tier materials. Excess T1/T2 becomes useful for endgame T3/T4 upgrades. Safety net for tight T3/T4 budgets.</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Material Conversion</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Chain Example</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>281 surplus T1 → ~93 T2 → ~31 T3 → ~10 T4. Covers shortfalls from aggressive upgrading.</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Material Sell</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Sell to Merchant</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>T1 = 5g, T2 = 15g, T3 = 40g, T4 = 100g, T5 = 250g. Emergency gold conversion. Deliberately poor exchange rate — upgrading is always better value.</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Storage Model</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Materials are NOT items. They do not count toward inventory threshold. Stored as 5 integer counters: T1_count through T5_count.</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Save Location</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>DataStore Key 2 (Inventory + Currencies) alongside gold. Minimal save space: 5 integers.</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>No Hard Cap</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>No maximum material count. Conversion sink and guild facility sink prevent unbounded hoarding.</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Guild Facility Sink</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Some guild facility levels require materials alongside gold. Specific tiers and quantities TBD per facility during Slice 8 design.</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Locked direction — details pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>UI Presentation</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Inventory Display</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Shown as 5 colored crystal/gem icons with count. Color-coded: Gray (T1), Green (T2), Blue (T3), Purple (T4), Gold (T5).</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Locked — Slice 7 presentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>UI Presentation</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Blacksmith Preview</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Shown in upgrade cost preview alongside gold: e.g. 'Cost: 1,170g + 10× Polished Core'.</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>Locked — Slice 7 presentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>UI Presentation</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Reward Preview</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Shown in quest/dispatch reward preview alongside gold and items.</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Locked — Slice 7 presentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>Simulation Benchmarks</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Lifetime Income (L1→L99)</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>T1: ~286, T2: ~286, T3: ~286, T4: ~286, T5: ~312 (includes daily events). Total ~1,456 materials.</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>Simulation Benchmarks</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Realistic Spend (10 upgrades)</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>T1: 5, T2: 100, T3: 255, T4: 255, T5: 55. Total 670 materials.</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>Simulation Benchmarks</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>T3/T4 Budget</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>89% used on realistic 10-upgrade scenario. Tight but positive with conversion safety net. Aggressive upgraders (10+ items) need targeted farming or conversion.</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>Simulation Benchmarks</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Design Feel</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Gold remains primary constraint. Materials are secondary — tight at T3/T4, comfortable at T1/T2, daily-gated at T5. Materials add a second resource axis without replacing gold as primary sink.</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Verified</t>
         </is>
       </c>
     </row>

</xml_diff>